<commit_message>
Improve summary template row styling
</commit_message>
<xml_diff>
--- a/weekly_summary_layout_template.xlsx
+++ b/weekly_summary_layout_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrewfarrell/Desktop/muckspreading-app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1191F1CC-EFA2-C14E-B35C-776A7726989E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C601AD32-280E-BF42-BBE9-C199722ED156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -587,7 +587,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -717,15 +717,6 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -776,13 +767,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
@@ -1230,7 +1220,7 @@
     </row>
     <row r="9" spans="1:6" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1324,7 +1314,7 @@
         <v>18.3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>14</v>
       </c>
@@ -1339,7 +1329,7 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="5" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1434,21 +1424,21 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5">
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4">
         <v>138.6</v>
       </c>
-      <c r="F26" s="5">
+      <c r="F26" s="4">
         <v>115.6</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="5" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1543,21 +1533,21 @@
       </c>
     </row>
     <row r="35" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5">
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4">
         <v>141.6</v>
       </c>
-      <c r="F35" s="5">
+      <c r="F35" s="4">
         <v>117.9</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="5" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1652,21 +1642,21 @@
       </c>
     </row>
     <row r="44" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B44" s="5"/>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5">
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4">
         <v>120</v>
       </c>
-      <c r="F44" s="5">
+      <c r="F44" s="4">
         <v>99.9</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A46" s="6" t="s">
+      <c r="A46" s="5" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1761,16 +1751,16 @@
       </c>
     </row>
     <row r="53" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="5" t="s">
+      <c r="A53" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B53" s="5"/>
-      <c r="C53" s="5"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="5">
+      <c r="B53" s="4"/>
+      <c r="C53" s="4"/>
+      <c r="D53" s="4"/>
+      <c r="E53" s="4">
         <v>160.30000000000001</v>
       </c>
-      <c r="F53" s="5">
+      <c r="F53" s="4">
         <v>133.5</v>
       </c>
     </row>
@@ -1865,16 +1855,16 @@
       </c>
     </row>
     <row r="61" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="5" t="s">
+      <c r="A61" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B61" s="5"/>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5"/>
-      <c r="E61" s="5">
+      <c r="B61" s="4"/>
+      <c r="C61" s="4"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4">
         <v>98.5</v>
       </c>
-      <c r="F61" s="5">
+      <c r="F61" s="4">
         <v>82</v>
       </c>
     </row>
@@ -1969,16 +1959,16 @@
       </c>
     </row>
     <row r="69" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="5" t="s">
+      <c r="A69" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B69" s="5"/>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5"/>
-      <c r="E69" s="5">
+      <c r="B69" s="4"/>
+      <c r="C69" s="4"/>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4">
         <v>141.5</v>
       </c>
-      <c r="F69" s="5">
+      <c r="F69" s="4">
         <v>117.99999999999999</v>
       </c>
     </row>
@@ -2073,21 +2063,21 @@
       </c>
     </row>
     <row r="77" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="5" t="s">
+      <c r="A77" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B77" s="5"/>
-      <c r="C77" s="5"/>
-      <c r="D77" s="5"/>
-      <c r="E77" s="5">
+      <c r="B77" s="4"/>
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4">
         <v>141.6</v>
       </c>
-      <c r="F77" s="5">
+      <c r="F77" s="4">
         <v>117.9</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A79" s="6" t="s">
+      <c r="A79" s="5" t="s">
         <v>42</v>
       </c>
     </row>
@@ -2165,21 +2155,21 @@
       </c>
     </row>
     <row r="85" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="5" t="s">
+      <c r="A85" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B85" s="5"/>
-      <c r="C85" s="5"/>
-      <c r="D85" s="5"/>
-      <c r="E85" s="5">
+      <c r="B85" s="4"/>
+      <c r="C85" s="4"/>
+      <c r="D85" s="4"/>
+      <c r="E85" s="4">
         <v>92.2</v>
       </c>
-      <c r="F85" s="5">
+      <c r="F85" s="4">
         <v>76.800000000000011</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A87" s="6" t="s">
+      <c r="A87" s="5" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2257,16 +2247,16 @@
       </c>
     </row>
     <row r="93" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="5" t="s">
+      <c r="A93" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B93" s="5"/>
-      <c r="C93" s="5"/>
-      <c r="D93" s="5"/>
-      <c r="E93" s="5">
+      <c r="B93" s="4"/>
+      <c r="C93" s="4"/>
+      <c r="D93" s="4"/>
+      <c r="E93" s="4">
         <v>126.80000000000001</v>
       </c>
-      <c r="F93" s="5">
+      <c r="F93" s="4">
         <v>105.6</v>
       </c>
     </row>

</xml_diff>